<commit_message>
UPDATE: Add and consolidate tests for DECIMAL and BASE
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/MATH_AND_TRIGONOMETRY/BASE_DECIMAL.xlsx
+++ b/xlsx/tests/calc_tests/MATH_AND_TRIGONOMETRY/BASE_DECIMAL.xlsx
@@ -1,15 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11027"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B1F164-9789-49FE-B74D-B574DC9618FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBE90D82-3731-FC43-BD4A-EF8AB6AA078D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-7240" yWindow="-26680" windowWidth="21800" windowHeight="12980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE" sheetId="2" r:id="rId1"/>
     <sheet name="DECIMAL" sheetId="3" r:id="rId2"/>
+    <sheet name="issue_1618" sheetId="4" r:id="rId3"/>
+    <sheet name="issue_1611" sheetId="5" r:id="rId4"/>
+    <sheet name="issue_1613" sheetId="6" r:id="rId5"/>
+    <sheet name="issue_1617" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="157">
   <si>
     <t>Number</t>
   </si>
@@ -479,6 +483,30 @@
   </si>
   <si>
     <t>Round-trip of BASE output</t>
+  </si>
+  <si>
+    <t>Leading space should be ignored</t>
+  </si>
+  <si>
+    <t>Trailing spaces are not</t>
+  </si>
+  <si>
+    <t>Many leading spaces are also ignored</t>
+  </si>
+  <si>
+    <t>Min length above maximum</t>
+  </si>
+  <si>
+    <t>Min length as date serial (above maximum)</t>
+  </si>
+  <si>
+    <t>Empty string</t>
+  </si>
+  <si>
+    <t>Empty text cell</t>
+  </si>
+  <si>
+    <t>string with whitespaces</t>
   </si>
 </sst>
 </file>
@@ -526,7 +554,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -549,12 +577,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1"/>
@@ -563,6 +602,7 @@
     <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
@@ -867,17 +907,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{504C306B-F88D-4DF0-9932-54AE4A851237}">
   <dimension ref="A1:I114"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.265625" customWidth="1"/>
-    <col min="2" max="2" width="12.86328125" customWidth="1"/>
-    <col min="3" max="3" width="11.53125" customWidth="1"/>
-    <col min="4" max="5" width="33.796875" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.5" customWidth="1"/>
+    <col min="4" max="5" width="33.83203125" customWidth="1"/>
     <col min="6" max="6" width="53.33203125" customWidth="1"/>
-    <col min="7" max="9" width="16.86328125" customWidth="1"/>
+    <col min="7" max="9" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -897,7 +937,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>10</v>
       </c>
@@ -916,7 +956,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>10</v>
       </c>
@@ -935,7 +975,7 @@
         <v>00001010</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>255</v>
       </c>
@@ -951,7 +991,7 @@
         <v>FF</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>255</v>
       </c>
@@ -970,7 +1010,7 @@
         <v>00FF</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>35</v>
       </c>
@@ -986,7 +1026,7 @@
         <v>Z</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>36</v>
       </c>
@@ -1002,7 +1042,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1018,7 +1058,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>16</v>
       </c>
@@ -1040,7 +1080,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>16</v>
       </c>
@@ -1062,7 +1102,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>16</v>
       </c>
@@ -1084,7 +1124,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>16</v>
       </c>
@@ -1106,7 +1146,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="D13" s="2" t="b">
         <f>ISNUMBER(_xlfn.BASE(16,7))</f>
         <v>0</v>
@@ -1119,7 +1159,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>10</v>
       </c>
@@ -1141,7 +1181,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>12345678</v>
       </c>
@@ -1163,7 +1203,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>1234</v>
       </c>
@@ -1182,7 +1222,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>23</v>
       </c>
@@ -1201,7 +1241,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>20</v>
       </c>
@@ -1220,7 +1260,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>123456789</v>
       </c>
@@ -1239,7 +1279,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>123456789</v>
       </c>
@@ -1258,7 +1298,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>0</v>
       </c>
@@ -1277,7 +1317,7 @@
         <v>00000</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>10</v>
       </c>
@@ -1296,7 +1336,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>123</v>
       </c>
@@ -1315,7 +1355,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>10</v>
       </c>
@@ -1334,7 +1374,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>10</v>
       </c>
@@ -1353,7 +1393,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>123456789</v>
       </c>
@@ -1372,7 +1412,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>40</v>
       </c>
@@ -1391,7 +1431,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>123456789</v>
       </c>
@@ -1410,7 +1450,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>10</v>
       </c>
@@ -1426,7 +1466,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>10</v>
       </c>
@@ -1442,7 +1482,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>10</v>
       </c>
@@ -1461,7 +1501,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>10</v>
       </c>
@@ -1477,7 +1517,7 @@
         <v>A</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>10</v>
       </c>
@@ -1493,7 +1533,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>20</v>
       </c>
@@ -1512,7 +1552,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>10.9</v>
       </c>
@@ -1531,7 +1571,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>12.567</v>
       </c>
@@ -1553,7 +1593,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>123.45677999999999</v>
       </c>
@@ -1572,7 +1612,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>-1</v>
       </c>
@@ -1591,7 +1631,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>-123456</v>
       </c>
@@ -1610,7 +1650,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>1000000000000000</v>
       </c>
@@ -1626,7 +1666,7 @@
         <v>11100011010111111010100100110001101000000000000000</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>10</v>
       </c>
@@ -1642,7 +1682,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <f>2^53-1</f>
         <v>9007199254740991</v>
@@ -1662,7 +1702,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <f>2^53-1</f>
         <v>9007199254740991</v>
@@ -1679,7 +1719,7 @@
         <v>2GOSA7PA2GV</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>5</v>
       </c>
@@ -1701,7 +1741,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>5</v>
       </c>
@@ -1723,7 +1763,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>5</v>
       </c>
@@ -1745,7 +1785,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>5</v>
       </c>
@@ -1767,7 +1807,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>255</v>
       </c>
@@ -1789,7 +1829,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>10</v>
       </c>
@@ -1805,7 +1845,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>33</v>
       </c>
@@ -1824,7 +1864,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>10</v>
       </c>
@@ -1840,7 +1880,7 @@
         <v>A</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>10</v>
       </c>
@@ -1859,7 +1899,7 @@
         <v>00001010</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" t="b">
         <v>1</v>
       </c>
@@ -1875,7 +1915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>10</v>
       </c>
@@ -1894,7 +1934,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>5</v>
       </c>
@@ -1913,7 +1953,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>37</v>
       </c>
@@ -1932,7 +1972,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>10</v>
       </c>
@@ -1948,7 +1988,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>5</v>
       </c>
@@ -1967,7 +2007,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
         <v>41</v>
       </c>
@@ -1986,7 +2026,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
         <v>42</v>
       </c>
@@ -2005,7 +2045,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
         <v>7</v>
       </c>
@@ -2024,7 +2064,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62">
         <f>DATE(2026,1,1)</f>
         <v>46023</v>
@@ -2044,7 +2084,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" t="e">
         <f>NA()</f>
         <v>#N/A</v>
@@ -2064,7 +2104,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>10</v>
       </c>
@@ -2084,7 +2124,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>10</v>
       </c>
@@ -2107,7 +2147,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" t="e">
         <f>1/0</f>
         <v>#DIV/0!</v>
@@ -2128,7 +2168,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>10</v>
       </c>
@@ -2152,7 +2192,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>10</v>
       </c>
@@ -2171,7 +2211,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>10</v>
       </c>
@@ -2187,7 +2227,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>10</v>
       </c>
@@ -2206,7 +2246,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>10</v>
       </c>
@@ -2222,7 +2262,7 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>10</v>
       </c>
@@ -2241,7 +2281,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>10</v>
       </c>
@@ -2257,7 +2297,7 @@
         <v>A</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>10</v>
       </c>
@@ -2276,7 +2316,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>10</v>
       </c>
@@ -2295,7 +2335,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>10</v>
       </c>
@@ -2314,7 +2354,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>10</v>
       </c>
@@ -2333,7 +2373,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>10</v>
       </c>
@@ -2352,7 +2392,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>10</v>
       </c>
@@ -2371,7 +2411,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>10</v>
       </c>
@@ -2390,7 +2430,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>10</v>
       </c>
@@ -2410,7 +2450,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>10</v>
       </c>
@@ -2430,7 +2470,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>10</v>
       </c>
@@ -2450,7 +2490,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>10</v>
       </c>
@@ -2470,7 +2510,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>5</v>
       </c>
@@ -2492,7 +2532,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>5</v>
       </c>
@@ -2511,7 +2551,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>5</v>
       </c>
@@ -2530,7 +2570,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>5</v>
       </c>
@@ -2552,7 +2592,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>5</v>
       </c>
@@ -2571,7 +2611,7 @@
         <v>000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000101</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>5</v>
       </c>
@@ -2593,7 +2633,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>0</v>
       </c>
@@ -2615,7 +2655,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>5</v>
       </c>
@@ -2637,7 +2677,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>5</v>
       </c>
@@ -2659,7 +2699,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>5</v>
       </c>
@@ -2681,7 +2721,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>5</v>
       </c>
@@ -2703,7 +2743,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>5</v>
       </c>
@@ -2725,7 +2765,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>5</v>
       </c>
@@ -2747,7 +2787,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>5</v>
       </c>
@@ -2770,7 +2810,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>5</v>
       </c>
@@ -2793,7 +2833,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>10</v>
       </c>
@@ -2816,7 +2856,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>10</v>
       </c>
@@ -2838,7 +2878,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D102" s="2" t="str">
         <f>_xlfn.BASE(10,"16")</f>
         <v>A</v>
@@ -2851,7 +2891,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D103" s="2" t="e">
         <f>_xlfn.BASE(10,TRUE)</f>
         <v>#NUM!</v>
@@ -2864,7 +2904,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D104" s="2" t="str">
         <f>_xlfn.BASE(TRUE,2)</f>
         <v>1</v>
@@ -2877,7 +2917,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D105" s="2" t="str">
         <f>_xlfn.BASE("255","16")</f>
         <v>FF</v>
@@ -2890,7 +2930,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D106" s="2" t="e">
         <f>_xlfn.BASE(255,H109:H112)</f>
         <v>#VALUE!</v>
@@ -2903,7 +2943,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D107" s="2" t="e">
         <f>_xlfn.BASE(G107:I107,2)</f>
         <v>#VALUE!</v>
@@ -2925,7 +2965,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D108" s="2" t="e">
         <f>_xlfn.BASE(G109:H112,2)</f>
         <v>#VALUE!</v>
@@ -2938,7 +2978,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D109" s="2" t="str">
         <f>_xlfn.BASE(G109:G112,2)</f>
         <v>1010</v>
@@ -2960,7 +3000,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D110" s="2" t="str">
         <f>_xlfn.BASE(255,H109:H112)</f>
         <v>FF</v>
@@ -2982,7 +3022,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D111" s="2" t="str">
         <f>_xlfn.BASE(G109:G112,H109:H112)</f>
         <v>7</v>
@@ -3004,7 +3044,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.2">
       <c r="E112" s="2" t="str">
         <f>_xlfn.BASE(5,2,I109:I112)</f>
         <v>000101</v>
@@ -3022,7 +3062,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="113" spans="4:6" x14ac:dyDescent="0.45">
+    <row r="113" spans="4:6" x14ac:dyDescent="0.2">
       <c r="D113" s="2" t="e">
         <f>_xlfn.BASE(G109:G112,2)</f>
         <v>#VALUE!</v>
@@ -3035,7 +3075,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="114" spans="4:6" x14ac:dyDescent="0.45">
+    <row r="114" spans="4:6" x14ac:dyDescent="0.2">
       <c r="E114" s="2" t="e">
         <f>_xlfn.BASE(5,2,I109:I112)</f>
         <v>#VALUE!</v>
@@ -3052,16 +3092,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8238C2D8-4264-4A7B-B498-1F42C76511D0}">
   <dimension ref="A1:I87"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.1328125" customWidth="1"/>
-    <col min="2" max="2" width="12.9296875" customWidth="1"/>
-    <col min="3" max="3" width="19.53125" customWidth="1"/>
+    <col min="1" max="1" width="23.1640625" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="19.5" customWidth="1"/>
     <col min="4" max="4" width="53.33203125" customWidth="1"/>
-    <col min="7" max="9" width="16.86328125" customWidth="1"/>
+    <col min="7" max="9" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>49</v>
       </c>
@@ -3076,7 +3116,7 @@
       </c>
       <c r="I1" s="3"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>51</v>
       </c>
@@ -3091,7 +3131,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>52</v>
       </c>
@@ -3103,7 +3143,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>53</v>
       </c>
@@ -3115,7 +3155,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>54</v>
       </c>
@@ -3127,7 +3167,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>55</v>
       </c>
@@ -3139,7 +3179,7 @@
         <v>1295</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>56</v>
       </c>
@@ -3154,7 +3194,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>57</v>
       </c>
@@ -3169,7 +3209,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>59</v>
       </c>
@@ -3184,7 +3224,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>61</v>
       </c>
@@ -3196,7 +3236,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="str">
         <f>_xlfn.BASE(16,10)</f>
         <v>16</v>
@@ -3212,7 +3252,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="str">
         <f>_xlfn.BASE(16,8)</f>
         <v>20</v>
@@ -3225,7 +3265,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="str">
         <f>_xlfn.BASE(16,4)</f>
         <v>100</v>
@@ -3238,7 +3278,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="str">
         <f>_xlfn.BASE(16,7)</f>
         <v>22</v>
@@ -3251,7 +3291,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="str">
         <f>_xlfn.BASE(10,16)</f>
         <v>A</v>
@@ -3264,7 +3304,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="str">
         <f>_xlfn.BASE(12345678,16)</f>
         <v>BC614E</v>
@@ -3277,7 +3317,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="str">
         <f>_xlfn.BASE(12.567,2)</f>
         <v>1100</v>
@@ -3290,7 +3330,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="e">
         <f>_xlfn.BASE(-123456,16)</f>
         <v>#NUM!</v>
@@ -3303,7 +3343,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="e">
         <f>_xlfn.BASE(-1,2)</f>
         <v>#NUM!</v>
@@ -3316,7 +3356,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="str">
         <f>_xlfn.BASE(123.45678,16)</f>
         <v>7B</v>
@@ -3329,7 +3369,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="str">
         <f>_xlfn.BASE(1234,2)</f>
         <v>10011010010</v>
@@ -3342,7 +3382,7 @@
         <v>1234</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="e">
         <f>_xlfn.BASE(123,1)</f>
         <v>#NUM!</v>
@@ -3355,7 +3395,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="str">
         <f>_xlfn.BASE(20,10.9)</f>
         <v>20</v>
@@ -3368,7 +3408,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="str">
         <f>_xlfn.BASE(20,11)</f>
         <v>19</v>
@@ -3381,7 +3421,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="str">
         <f>_xlfn.BASE(23,3)</f>
         <v>212</v>
@@ -3394,7 +3434,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="str">
         <f>_xlfn.BASE(123456789,9)</f>
         <v>277266780</v>
@@ -3407,7 +3447,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="e">
         <f>_xlfn.BASE(123456789,45)</f>
         <v>#NUM!</v>
@@ -3420,7 +3460,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="str">
         <f>_xlfn.BASE(123456789,36)</f>
         <v>21I3V9</v>
@@ -3433,7 +3473,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="e">
         <f>_xlfn.BASE(123456789,37)</f>
         <v>#NUM!</v>
@@ -3446,7 +3486,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="e">
         <f>_xlfn.BASE(40,37)</f>
         <v>#NUM!</v>
@@ -3459,7 +3499,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>1</v>
       </c>
@@ -3474,7 +3514,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>33</v>
       </c>
@@ -3489,7 +3529,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>33</v>
       </c>
@@ -3504,7 +3544,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>33</v>
       </c>
@@ -3516,7 +3556,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>33</v>
       </c>
@@ -3528,7 +3568,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>33</v>
       </c>
@@ -3543,7 +3583,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>33</v>
       </c>
@@ -3555,7 +3595,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>33</v>
       </c>
@@ -3567,7 +3607,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>42</v>
       </c>
@@ -3582,7 +3622,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>64</v>
       </c>
@@ -3597,7 +3637,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>66</v>
       </c>
@@ -3612,7 +3652,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="str">
         <f>REPT("1",53)</f>
         <v>11111111111111111111111111111111111111111111111111111</v>
@@ -3628,7 +3668,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="str">
         <f>REPT("0",254)&amp;"1"</f>
         <v>000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000001</v>
@@ -3644,7 +3684,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>33</v>
       </c>
@@ -3656,7 +3696,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>101</v>
       </c>
@@ -3671,7 +3711,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46">
         <f>DATE(2026,1,1)</f>
         <v>46023</v>
@@ -3687,7 +3727,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="b">
         <v>1</v>
       </c>
@@ -3702,7 +3742,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="b">
         <v>0</v>
       </c>
@@ -3714,7 +3754,7 @@
         <v>25689038</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>33</v>
       </c>
@@ -3729,7 +3769,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>33</v>
       </c>
@@ -3744,7 +3784,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>33</v>
       </c>
@@ -3759,7 +3799,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>33</v>
       </c>
@@ -3774,7 +3814,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="e">
         <f>NA()</f>
         <v>#N/A</v>
@@ -3790,7 +3830,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>33</v>
       </c>
@@ -3806,7 +3846,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="e">
         <f>1/0</f>
         <v>#DIV/0!</v>
@@ -3823,7 +3863,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>33</v>
       </c>
@@ -3838,7 +3878,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
         <v>33</v>
       </c>
@@ -3850,7 +3890,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
         <v>33</v>
       </c>
@@ -3865,7 +3905,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
         <v>33</v>
       </c>
@@ -3877,7 +3917,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
         <v>33</v>
       </c>
@@ -3892,7 +3932,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
         <v>33</v>
       </c>
@@ -3904,7 +3944,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
         <v>33</v>
       </c>
@@ -3919,7 +3959,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
         <v>33</v>
       </c>
@@ -3934,7 +3974,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" s="4" t="s">
         <v>33</v>
       </c>
@@ -3949,7 +3989,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
         <v>33</v>
       </c>
@@ -3964,7 +4004,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
         <v>33</v>
       </c>
@@ -3979,7 +4019,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
         <v>33</v>
       </c>
@@ -3994,7 +4034,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
         <v>33</v>
       </c>
@@ -4010,7 +4050,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" s="4" t="s">
         <v>33</v>
       </c>
@@ -4026,7 +4066,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
         <v>122</v>
       </c>
@@ -4041,7 +4081,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
         <v>33</v>
       </c>
@@ -4057,7 +4097,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
         <v>33</v>
       </c>
@@ -4073,7 +4113,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
         <v>62</v>
       </c>
@@ -4088,7 +4128,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
         <v>62</v>
       </c>
@@ -4103,7 +4143,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C75" s="2" t="e">
         <f>_xlfn.DECIMAL("FF",TRUE)</f>
         <v>#NUM!</v>
@@ -4112,7 +4152,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C76" s="2">
         <f>_xlfn.DECIMAL("FF","1.6E1")</f>
         <v>255</v>
@@ -4121,7 +4161,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C77" s="2">
         <f>_xlfn.DECIMAL(TRUE,36)</f>
         <v>1389110</v>
@@ -4130,7 +4170,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C78" s="2">
         <f>_xlfn.DECIMAL(101,2)</f>
         <v>5</v>
@@ -4139,7 +4179,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C79" s="2">
         <f>_xlfn.DECIMAL("FF","16")</f>
         <v>255</v>
@@ -4148,7 +4188,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C80" s="2" t="e">
         <f>_xlfn.DECIMAL("FF",H83:H86)</f>
         <v>#VALUE!</v>
@@ -4157,7 +4197,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="81" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="81" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C81" s="2" t="e">
         <f>_xlfn.DECIMAL(G81:H81,16)</f>
         <v>#VALUE!</v>
@@ -4172,7 +4212,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="82" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="82" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C82" s="2" t="e">
         <f>_xlfn.DECIMAL(G83:H86,16)</f>
         <v>#VALUE!</v>
@@ -4181,7 +4221,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="83" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="83" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C83" s="2">
         <f>_xlfn.DECIMAL(G83:G86,2)</f>
         <v>10</v>
@@ -4196,7 +4236,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="84" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C84" s="2">
         <f>_xlfn.DECIMAL("FF",H83:H86)</f>
         <v>255</v>
@@ -4211,7 +4251,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="85" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="85" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C85" s="2">
         <f>_xlfn.DECIMAL(G83:G86,H83:H86)</f>
         <v>511</v>
@@ -4226,7 +4266,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="86" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="86" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C86" s="2">
         <f>_xlfn.DECIMAL(G83:G86,H83:H86)</f>
         <v>35</v>
@@ -4241,13 +4281,353 @@
         <v>36</v>
       </c>
     </row>
-    <row r="87" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="87" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C87" s="2" t="e">
         <f>_xlfn.DECIMAL(G83:G86,16)</f>
         <v>#VALUE!</v>
       </c>
       <c r="D87" t="s">
         <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{230A06E5-843F-9F4D-9697-FFF9F07D35DB}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2">
+        <f>_xlfn.DECIMAL(A2,B2)</f>
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="str">
+        <f>" 10"</f>
+        <v xml:space="preserve"> 10</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2">
+        <f t="shared" ref="C3:C8" si="0">_xlfn.DECIMAL(A3,B3)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="str">
+        <f>" 10  "</f>
+        <v xml:space="preserve"> 10  </v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="e">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="D4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="str">
+        <f>"    10"</f>
+        <v xml:space="preserve">    10</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>10</v>
+      </c>
+      <c r="B6" t="str">
+        <f>"   2"</f>
+        <v xml:space="preserve">   2</v>
+      </c>
+      <c r="C6" s="2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>10</v>
+      </c>
+      <c r="B7" t="str">
+        <f>"2   "</f>
+        <v xml:space="preserve">2   </v>
+      </c>
+      <c r="C7" s="8">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>10</v>
+      </c>
+      <c r="B8" t="str">
+        <f>"   2  "</f>
+        <v xml:space="preserve">   2  </v>
+      </c>
+      <c r="C8" s="8">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA9B0045-236A-FF4A-932D-C2D317D357FD}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>-9.9999999999999995E-8</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="e">
+        <f>_xlfn.BASE(A2,B2)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="E2" s="2" t="e">
+        <f>_xlfn.BASE(A2,B2,C2)</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>-0.5</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="e">
+        <f>_xlfn.BASE(A3,B3)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="E3" s="2" t="e">
+        <f>_xlfn.BASE(A3,B3,C3)</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22EA525F-13FE-9B47-829A-38EA2CA55E9A}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>5</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>256</v>
+      </c>
+      <c r="D2" s="2" t="str">
+        <f>_xlfn.BASE(A2,B2)</f>
+        <v>101</v>
+      </c>
+      <c r="E2" s="2" t="e">
+        <f>_xlfn.BASE(A2,B2,C2)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="F2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <f>DATE(1910,1,8)</f>
+        <v>3661</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <f>_xlfn.BASE(A3,B3)</f>
+        <v>101</v>
+      </c>
+      <c r="E3" s="2" t="e">
+        <f>_xlfn.BASE(A3,B3,C3)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="F3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28F87FF4-D7E9-3D46-A705-BFB0082C693A}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2">
+        <f>_xlfn.DECIMAL(A2,B2)</f>
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2">
+        <f>_xlfn.DECIMAL(A3,B3)</f>
+        <v>0</v>
+      </c>
+      <c r="D3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="str">
+        <f>".  "</f>
+        <v xml:space="preserve">.  </v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="e">
+        <f>_xlfn.DECIMAL(A4,B4)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="D4" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE: Consolidate tests for DECIMAL
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/MATH_AND_TRIGONOMETRY/BASE_DECIMAL.xlsx
+++ b/xlsx/tests/calc_tests/MATH_AND_TRIGONOMETRY/BASE_DECIMAL.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11011"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBE90D82-3731-FC43-BD4A-EF8AB6AA078D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB72D435-65FB-3A41-87E7-4E6ED8CFBE99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-7240" yWindow="-26680" windowWidth="21800" windowHeight="12980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-7240" yWindow="-26680" windowWidth="21800" windowHeight="12980" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE" sheetId="2" r:id="rId1"/>
@@ -14,6 +14,8 @@
     <sheet name="issue_1611" sheetId="5" r:id="rId4"/>
     <sheet name="issue_1613" sheetId="6" r:id="rId5"/>
     <sheet name="issue_1617" sheetId="7" r:id="rId6"/>
+    <sheet name="issue_1615" sheetId="8" r:id="rId7"/>
+    <sheet name="issue_1616" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="163">
   <si>
     <t>Number</t>
   </si>
@@ -507,6 +509,24 @@
   </si>
   <si>
     <t>string with whitespaces</t>
+  </si>
+  <si>
+    <t>-10</t>
+  </si>
+  <si>
+    <t>Leading minus sign accepted as a sign</t>
+  </si>
+  <si>
+    <t>+10</t>
+  </si>
+  <si>
+    <t>Leading plus sign accepted as a sign</t>
+  </si>
+  <si>
+    <t>Number cast to text, leading minus sign accepted as a sign</t>
+  </si>
+  <si>
+    <t>Text length above maximum (255)</t>
   </si>
 </sst>
 </file>
@@ -4633,4 +4653,123 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9653A76C-D14F-A342-A350-3872413A6704}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.33203125" customWidth="1"/>
+    <col min="3" max="3" width="14.5" customWidth="1"/>
+    <col min="4" max="4" width="50.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="e">
+        <f>_xlfn.DECIMAL(A2,B2)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="D2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="e">
+        <f>_xlfn.DECIMAL(A3,B3)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="D3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>-5</v>
+      </c>
+      <c r="B4">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="e">
+        <f>_xlfn.DECIMAL(A4,B4)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="D4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF44F0BD-F3CF-0740-8FB1-079A0B842DB7}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="60.33203125" customWidth="1"/>
+    <col min="3" max="3" width="14.5" customWidth="1"/>
+    <col min="4" max="4" width="35.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="str">
+        <f>REPT("0",255)&amp;"1"</f>
+        <v>0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000001</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="e">
+        <f>_xlfn.DECIMAL(A2,B2)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>